<commit_message>
feat: connect frontend to Vercel backend API for comments/submissions/favorites
- Add LH_API_BASE to index.html and store.html for API connectivity
- Updated serverless APIs to use GitHub Issues as backend storage
- Images will be stored in images/ folder via GitHub API
</commit_message>
<xml_diff>
--- a/상점 리스트.xlsx
+++ b/상점 리스트.xlsx
@@ -2206,6 +2206,7 @@
         <color theme="1"/>
         <rFont val="Poppins"/>
         <family val="0"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -2215,6 +2216,7 @@
         <color theme="1"/>
         <rFont val="맑은 고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">주일 영업</t>
     </r>
@@ -3054,6 +3056,7 @@
         <color theme="1"/>
         <rFont val="Poppins"/>
         <family val="0"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -3063,6 +3066,7 @@
         <color theme="1"/>
         <rFont val="맑은 고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">주일 영업</t>
     </r>
@@ -4238,6 +4242,7 @@
         <color theme="1"/>
         <rFont val="Poppins"/>
         <family val="0"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">, </t>
     </r>
@@ -4247,6 +4252,7 @@
         <color theme="1"/>
         <rFont val="맑은 고딕"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">주일 영업</t>
     </r>
@@ -6552,7 +6558,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6618,18 +6624,6 @@
       <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Poppins"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="맑은 고딕"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -6722,79 +6716,79 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7054,790 +7048,790 @@
   <dimension ref="A3:M24"/>
   <sheetFormatPr defaultColWidth="8.6171875" defaultRowHeight="17.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="41.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="32.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="37.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="40.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="26.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="31.92"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="43.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="100.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="32.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="37.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="40.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="26.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="31.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="43.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="100.85"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="17.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1"/>
-      <c r="B3" s="2" t="s">
+      <c r="A3" s="2"/>
+      <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="M3" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="1" t="s">
+      <c r="D4" s="8"/>
+      <c r="E4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="K4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="L4" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="M4" s="9" t="s">
+      <c r="M4" s="10" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="1" t="s">
+      <c r="D5" s="8"/>
+      <c r="E5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="L5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="M5" s="10" t="s">
+      <c r="M5" s="11" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="1" t="s">
+      <c r="D6" s="8"/>
+      <c r="E6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="K6" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="L6" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="M6" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="11"/>
-      <c r="E7" s="1" t="s">
+      <c r="D7" s="12"/>
+      <c r="E7" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="K7" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="L7" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="M7" s="2" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="17.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="17.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
+    <row r="9" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="1" t="s">
+      <c r="D9" s="12"/>
+      <c r="E9" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="I9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="K9" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="L9" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="M9" s="1" t="s">
+      <c r="M9" s="2" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="D10" s="11"/>
-      <c r="E10" s="1" t="s">
+      <c r="D10" s="12"/>
+      <c r="E10" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="13" t="n">
         <v>12000</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="I10" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="K10" s="8" t="s">
+      <c r="K10" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="L10" s="1" t="s">
+      <c r="L10" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="M10" s="1" t="s">
+      <c r="M10" s="2" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D11" s="11"/>
-      <c r="E11" s="1" t="s">
+      <c r="D11" s="12"/>
+      <c r="E11" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="K11" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="L11" s="1" t="s">
+      <c r="L11" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="M11" s="1" t="s">
+      <c r="M11" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="17.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="n">
+    <row r="12" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="11"/>
-      <c r="E12" s="1" t="s">
+      <c r="D12" s="12"/>
+      <c r="E12" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="H12" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="I12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="J12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="K12" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="L12" s="1" t="s">
+      <c r="L12" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="M12" s="1" t="s">
+      <c r="M12" s="2" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D13" s="11"/>
-      <c r="E13" s="1" t="s">
+      <c r="D13" s="12"/>
+      <c r="E13" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="H13" s="8" t="s">
+      <c r="H13" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="I13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J13" s="8" t="s">
+      <c r="J13" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="K13" s="8" t="s">
+      <c r="K13" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="L13" s="1" t="s">
+      <c r="L13" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="M13" s="1" t="s">
+      <c r="M13" s="2" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="1" t="s">
+      <c r="D14" s="8"/>
+      <c r="E14" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="13" t="n">
         <v>14000</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="H14" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="I14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="J14" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K14" s="8" t="s">
+      <c r="K14" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="L14" s="1" t="s">
+      <c r="L14" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="M14" s="1" t="s">
+      <c r="M14" s="2" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D15" s="7"/>
-      <c r="E15" s="1" t="s">
+      <c r="D15" s="8"/>
+      <c r="E15" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="H15" s="8" t="s">
+      <c r="H15" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="I15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J15" s="1" t="s">
+      <c r="J15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="K15" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="L15" s="1" t="s">
+      <c r="L15" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="M15" s="1" t="s">
+      <c r="M15" s="2" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="47.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="7"/>
-      <c r="E16" s="1" t="s">
+      <c r="D16" s="8"/>
+      <c r="E16" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G16" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="I16" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J16" s="8" t="s">
+      <c r="J16" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="K16" s="8" t="s">
+      <c r="K16" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="L16" s="1" t="s">
+      <c r="L16" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="M16" s="1" t="s">
+      <c r="M16" s="2" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="1" t="s">
+      <c r="D17" s="14"/>
+      <c r="E17" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="G17" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="H17" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="I17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J17" s="1" t="s">
+      <c r="J17" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="K17" s="8" t="s">
+      <c r="K17" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="L17" s="1" t="s">
+      <c r="L17" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="M17" s="1" t="s">
+      <c r="M17" s="2" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="1" t="s">
+      <c r="D18" s="14"/>
+      <c r="E18" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="H18" s="8" t="s">
+      <c r="H18" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="I18" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="J18" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="K18" s="8" t="s">
+      <c r="K18" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="L18" s="1" t="s">
+      <c r="L18" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="M18" s="1" t="s">
+      <c r="M18" s="2" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="n">
+      <c r="A19" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D19" s="7"/>
-      <c r="E19" s="1" t="s">
+      <c r="D19" s="8"/>
+      <c r="E19" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="F19" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="G19" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="H19" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="I19" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J19" s="1" t="s">
+      <c r="J19" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="K19" s="8" t="s">
+      <c r="K19" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="L19" s="1" t="s">
+      <c r="L19" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="M19" s="1" t="s">
+      <c r="M19" s="2" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="n">
+      <c r="A20" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D20" s="13"/>
-      <c r="E20" s="1" t="s">
+      <c r="D20" s="14"/>
+      <c r="E20" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="F20" s="1"/>
-      <c r="G20" s="14" t="s">
+      <c r="F20" s="2"/>
+      <c r="G20" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="n">
+      <c r="A21" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="D21" s="13"/>
-      <c r="E21" s="1" t="s">
+      <c r="D21" s="14"/>
+      <c r="E21" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="F21" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="G21" s="10" t="s">
+      <c r="G21" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1" t="s">
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="M21" s="1" t="s">
+      <c r="M21" s="2" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="17.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="n">
+    <row r="22" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="13"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="15" t="s">
+      <c r="D22" s="14"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1" t="s">
+      <c r="D23" s="2"/>
+      <c r="E23" s="2" t="s">
         <v>160</v>
       </c>
       <c r="F23" s="17" t="s">
         <v>161</v>
       </c>
-      <c r="G23" s="1" t="s">
+      <c r="G23" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="H23" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="I23" s="1" t="s">
+      <c r="I23" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J23" s="1" t="s">
+      <c r="J23" s="2" t="s">
         <v>29</v>
       </c>
       <c r="K23" s="17" t="s">
         <v>163</v>
       </c>
-      <c r="L23" s="1" t="s">
+      <c r="L23" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="M23" s="1" t="s">
+      <c r="M23" s="2" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="n">
+      <c r="A24" s="7" t="n">
         <v>23.6666666666667</v>
       </c>
       <c r="B24" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1" t="s">
+      <c r="D24" s="2"/>
+      <c r="E24" s="2" t="s">
         <v>167</v>
       </c>
       <c r="F24" s="19" t="n">
@@ -7846,22 +7840,22 @@
       <c r="G24" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="H24" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="I24" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J24" s="1" t="s">
+      <c r="J24" s="2" t="s">
         <v>169</v>
       </c>
       <c r="K24" s="17" t="s">
         <v>170</v>
       </c>
-      <c r="L24" s="1" t="s">
+      <c r="L24" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="M24" s="1" t="s">
+      <c r="M24" s="2" t="s">
         <v>172</v>
       </c>
     </row>

</xml_diff>